<commit_message>
Add input templates for queries and responses
- Created new Excel file `2026-07-24T21-48-35-079Z-input-template.xlsx` with sample queries and responses.
- Created new Excel file `2026-07-30T03-00-49-474Z-input-template.xlsx` with updated queries and responses.
- Each file includes a structured format with metadata, styles, and themes for better usability.
</commit_message>
<xml_diff>
--- a/examples/input-template.xlsx
+++ b/examples/input-template.xlsx
@@ -404,7 +404,7 @@
         <v>query</v>
       </c>
       <c r="B1" t="str">
-        <v>reference_answer</v>
+        <v>response</v>
       </c>
     </row>
     <row r="2">
@@ -420,7 +420,7 @@
         <v>Explain REST APIs in one sentence.</v>
       </c>
       <c r="B3" t="str">
-        <v>REST APIs are HTTP interfaces that expose resources through standard methods like GET and POST.</v>
+        <v>REST APIs are interfaces that expose resources over HTTP methods.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>